<commit_message>
Add cleaned IPM and poverty data
</commit_message>
<xml_diff>
--- a/data/data-mentah/IPM_2022.xlsx
+++ b/data/data-mentah/IPM_2022.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{023A27B0-C60E-43F5-974B-2DBB34D4F6DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6DAF05-8944-411B-BEAF-7020A9EB0ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>Kabupaten/Kota</t>
   </si>
@@ -183,12 +183,6 @@
   </si>
   <si>
     <t>80.24</t>
-  </si>
-  <si>
-    <t>Sulawesi Selatan</t>
-  </si>
-  <si>
-    <t>73.96</t>
   </si>
 </sst>
 </file>
@@ -565,10 +559,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -576,7 +570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -584,7 +578,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -592,7 +586,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -600,7 +594,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -608,7 +602,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -616,7 +610,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -624,7 +618,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -632,7 +626,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -640,7 +634,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -648,7 +642,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -656,7 +650,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -664,7 +658,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -672,7 +666,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -680,7 +674,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -688,7 +682,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -696,7 +690,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -704,7 +698,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -712,7 +706,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -720,7 +714,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>38</v>
       </c>
@@ -728,7 +722,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>40</v>
       </c>
@@ -736,7 +730,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>42</v>
       </c>
@@ -744,7 +738,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>44</v>
       </c>
@@ -752,7 +746,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>46</v>
       </c>
@@ -760,26 +754,18 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>48</v>
       </c>
       <c r="B25" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:H27" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:H26" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>